<commit_message>
backbone_c correction per Fischer/Zamboni + audit fixes
LabelledCompound now takes backbone_c so the natural-abundance correction
only uses derivative carbons. Also fixes mdv_AA element-wise math, the
file_parser ExcelWriter overwriting each sheet, and UI wiring.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -1,32 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="alanine_M_57" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="pyruvate_M_57" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="citrate_M_57" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -45,13 +49,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -339,10 +410,316 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>1.2547</v>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>-0.2041</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1.2547</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>-0.0658</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.2041</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.2547</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.0163</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.0658</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-0.2041</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.2547</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>1.1339</v>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>-0.1014</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1.1339</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>-0.0387</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.1014</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.1339</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.0056</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.0387</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-0.1014</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.1339</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>1.5107</v>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>-0.4691</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1.5107</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>-0.0791</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.4691</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.5107</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.0791</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-0.4691</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.5107</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.0791</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.4691</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.5107</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.0791</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.4691</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.5107</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.0791</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.4691</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.5107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
sum multi-isotope combos in valid_combos; pin tests to Nanchen 2007
valid_combos previously returned only the first combination summing to the
target mass shift. For elements with >=3 isotopes (O, Si, S, Cl, Br), multiple
combos share the same mass shift and must all be summed - this is explicit in
Nanchen et al. 2007 Fig. Si correction matrix (Si28*Si30 + Si29^2).

Correction matrix for the alanine (M-57)+ worked example now matches the
paper's published values to 4 decimal places.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -420,7 +420,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>1.2547</v>
+        <v>1.2963</v>
       </c>
       <c r="B1" t="n">
         <v>0</v>
@@ -434,10 +434,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-0.2041</v>
+        <v>-0.2535</v>
       </c>
       <c r="B2" t="n">
-        <v>1.2547</v>
+        <v>1.2963</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -448,13 +448,13 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-0.0658</v>
+        <v>-0.0635</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.2041</v>
+        <v>-0.2535</v>
       </c>
       <c r="C3" t="n">
-        <v>1.2547</v>
+        <v>1.2963</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -462,16 +462,16 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.0163</v>
+        <v>0.0199</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.0658</v>
+        <v>-0.0635</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.2041</v>
+        <v>-0.2535</v>
       </c>
       <c r="D4" t="n">
-        <v>1.2547</v>
+        <v>1.2963</v>
       </c>
     </row>
   </sheetData>
@@ -490,7 +490,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>1.1339</v>
+        <v>1.1338</v>
       </c>
       <c r="B1" t="n">
         <v>0</v>
@@ -507,7 +507,7 @@
         <v>-0.1014</v>
       </c>
       <c r="B2" t="n">
-        <v>1.1339</v>
+        <v>1.1338</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -518,13 +518,13 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-0.0387</v>
+        <v>-0.0388</v>
       </c>
       <c r="B3" t="n">
         <v>-0.1014</v>
       </c>
       <c r="C3" t="n">
-        <v>1.1339</v>
+        <v>1.1338</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -535,13 +535,13 @@
         <v>0.0056</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.0387</v>
+        <v>-0.0388</v>
       </c>
       <c r="C4" t="n">
         <v>-0.1014</v>
       </c>
       <c r="D4" t="n">
-        <v>1.1339</v>
+        <v>1.1338</v>
       </c>
     </row>
   </sheetData>
@@ -583,7 +583,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>-0.4691</v>
+        <v>-0.4692</v>
       </c>
       <c r="B2" t="n">
         <v>1.5107</v>
@@ -606,10 +606,10 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-0.0791</v>
+        <v>-0.0906</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.4691</v>
+        <v>-0.4692</v>
       </c>
       <c r="C3" t="n">
         <v>1.5107</v>
@@ -629,13 +629,13 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.0457</v>
+        <v>0.0508</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.0791</v>
+        <v>-0.0906</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.4691</v>
+        <v>-0.4692</v>
       </c>
       <c r="D4" t="n">
         <v>1.5107</v>
@@ -652,16 +652,16 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.0007</v>
+        <v>0.0014</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0457</v>
+        <v>0.0508</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.0791</v>
+        <v>-0.0906</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.4691</v>
+        <v>-0.4692</v>
       </c>
       <c r="E5" t="n">
         <v>1.5107</v>
@@ -675,19 +675,19 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>-0.0025</v>
+        <v>-0.0033</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0007</v>
+        <v>0.0014</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0457</v>
+        <v>0.0508</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0791</v>
+        <v>-0.0906</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.4691</v>
+        <v>-0.4692</v>
       </c>
       <c r="F6" t="n">
         <v>1.5107</v>
@@ -701,19 +701,19 @@
         <v>0.0002</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.0025</v>
+        <v>-0.0033</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0007</v>
+        <v>0.0014</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0457</v>
+        <v>0.0508</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0791</v>
+        <v>-0.0906</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.4691</v>
+        <v>-0.4692</v>
       </c>
       <c r="G7" t="n">
         <v>1.5107</v>

</xml_diff>